<commit_message>
Replace Jessica (home-only) with Le Salon Vagabond in seeding list
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -571,32 +571,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>@jessicalacoiffureatonimage</t>
+          <t>@lesalonvagabond</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>52 Chemin des Rousselles, 69640 Lacenas</t>
+          <t>4 Grand Rue, 34725 Saint-André-de-Sangonis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>La Coiffure à ton image</t>
+          <t>Le Salon Vagabond</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Coiffeuse-maquilleuse mariée + formatrice</t>
+          <t>Coloriste blond polaire / balayage + formatrice</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JESSICA</t>
+          <t>VAGABOND</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers coiffure et maquillage mariée, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Marion 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond polaire et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est VAGABOND. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep Jessica (already contacted) and add Le Salon Vagabond: 34 seeding contacts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -603,465 +603,465 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>@formation.graziella.debousse</t>
+          <t>@jessicalacoiffureatonimage</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28 allée CF Justin Josserand, 26200 Montélimar</t>
+          <t>52 Chemin des Rousselles, 69640 Lacenas (à domicile)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Institut de Formation GD</t>
+          <t>La Coiffure à ton image</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Coiffeuse + directrice/formatrice</t>
+          <t>Coiffeuse-maquilleuse mariée À DOMICILE + formatrice (déjà contactée)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GRAZIELLA</t>
+          <t>JESSICA</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Graziella 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours et votre travail de formatrice, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est GRAZIELLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers coiffure et maquillage mariée, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>@kosmocut_hairstyl (à confirmer)</t>
+          <t>@formation.graziella.debousse</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>20 rue de l'Horloge, 63200 Riom</t>
+          <t>28 allée CF Justin Josserand, 26200 Montélimar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Synergie Coiffure Esthétique</t>
+          <t>Institut de Formation GD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Coiffeuse championne du monde + formatrice</t>
+          <t>Coiffeuse + directrice/formatrice</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LISA</t>
+          <t>GRAZIELLA</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Graziella 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours et votre travail de formatrice, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est GRAZIELLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>@oceaneavakian</t>
+          <t>@kosmocut_hairstyl (à confirmer)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32 rue Cuvier, 69006 Lyon</t>
+          <t>20 rue de l'Horloge, 63200 Riom</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Salon Océane Avakian</t>
+          <t>Synergie Coiffure Esthétique</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Coloriste balayage + formatrice</t>
+          <t>Coiffeuse championne du monde + formatrice</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OCEANE</t>
+          <t>LISA</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Océane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et vos formations, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OCEANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>@thomastuccinardi</t>
+          <t>@oceaneavakian</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>39 rue de la République, 69002 Lyon</t>
+          <t>32 rue Cuvier, 69006 Lyon</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thomas Tuccinardi</t>
+          <t>Salon Océane Avakian</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Coloriste expert + formateur (Redken)</t>
+          <t>Coloriste balayage + formatrice</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>THOMAS</t>
+          <t>OCEANE</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Thomas 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Océane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et vos formations, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OCEANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>@yohanmenzoyan</t>
+          <t>@thomastuccinardi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>37 Corniche de Solviou, 83140 Six-Fours-les-Plages</t>
+          <t>39 rue de la République, 69002 Lyon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The Hairdresser</t>
+          <t>Thomas Tuccinardi</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Coiffeur/gérant + formateur</t>
+          <t>Coloriste expert + formateur (Redken)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>YOHAN</t>
+          <t>THOMAS</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yohan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre vision du métier et vos salons, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YOHAN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Thomas 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>@backstage_by_karatas</t>
+          <t>@yohanmenzoyan</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>89 rue des Grandes Arcades, 67000 Strasbourg</t>
+          <t>37 Corniche de Solviou, 83140 Six-Fours-les-Plages</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Backstage by Karatas</t>
+          <t>The Hairdresser</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Coloriste balayage/blond + formatrice (ALSACE)</t>
+          <t>Coiffeur/gérant + formateur</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AYLA</t>
+          <t>YOHAN</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Ayla 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est AYLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Yohan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre vision du métier et vos salons, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YOHAN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>@sibelhairartist</t>
+          <t>@backstage_by_karatas</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14 Avenue de Strasbourg, 67170 Brumath</t>
+          <t>89 rue des Grandes Arcades, 67000 Strasbourg</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sibel Hair Artist</t>
+          <t>Backstage by Karatas</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Coloriste balayage + formatrice (ALSACE)</t>
+          <t>Coloriste balayage/blond + formatrice (ALSACE)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SIBEL</t>
+          <t>AYLA</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sibel 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SIBEL. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Ayla 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est AYLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>@lamaisonducoloriste</t>
+          <t>@sibelhairartist</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>18 rue des Ponts de Comines, 59800 Lille</t>
+          <t>14 Avenue de Strasbourg, 67170 Brumath</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>La Maison du Coloriste</t>
+          <t>Sibel Hair Artist</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Coloriste + formateur</t>
+          <t>Coloriste balayage + formatrice (ALSACE)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEBASTIEN</t>
+          <t>SIBEL</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sébastien 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre approche du métier de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SEBASTIEN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sibel 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SIBEL. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>@l.atypique</t>
+          <t>@lamaisonducoloriste</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16 rue Littré, 75006 Paris</t>
+          <t>18 rue des Ponts de Comines, 59800 Lille</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>L.Atypique</t>
+          <t>La Maison du Coloriste</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Coloriste blond/balayage + formatrice</t>
+          <t>Coloriste + formateur</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LATYPIQUE</t>
+          <t>SEBASTIEN</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mélanie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LATYPIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sébastien 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre approche du métier de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SEBASTIEN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>@brookelynbalayage</t>
+          <t>@l.atypique</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9 Place Carnot, 69002 Lyon</t>
+          <t>16 rue Littré, 75006 Paris</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CL Concept</t>
+          <t>L.Atypique</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Coloriste AirTouch + formatrice</t>
+          <t>Coloriste blond/balayage + formatrice</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BROOKELYN</t>
+          <t>LATYPIQUE</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Bonjour BrookeLyn 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du balayage AirTouch, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est BROOKELYN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Mélanie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LATYPIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>@salon_kf</t>
+          <t>@brookelynbalayage</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>69 Bd Ernest Dalby, 44000 Nantes</t>
+          <t>9 Place Carnot, 69002 Lyon</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Salon KF</t>
+          <t>CL Concept</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Coiffeur coloriste + formateur</t>
+          <t>Coloriste AirTouch + formatrice</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SALONKF</t>
+          <t>BROOKELYN</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Kévin 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SALONKF. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour BrookeLyn 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du balayage AirTouch, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est BROOKELYN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>@olivierlebrun_paris</t>
+          <t>@salon_kf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>5 bis rue du Louvre, 75001 Paris</t>
+          <t>69 Bd Ernest Dalby, 44000 Nantes</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OLAB Paris</t>
+          <t>Salon KF</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hairstylist studio + formateur (à confirmer)</t>
+          <t>Coiffeur coloriste + formateur</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OLIVIER</t>
+          <t>SALONKF</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Olivier 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers hairstyle, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OLIVIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Kévin 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SALONKF. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>@yassine.jarrar</t>
+          <t>@olivierlebrun_paris</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>21 Parvis Saint-Maurice, 59000 Lille</t>
+          <t>5 bis rue du Louvre, 75001 Paris</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Les Vilains Barber</t>
+          <t>OLAB Paris</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Barbier + formateur (LVB Formation)</t>
+          <t>Hairstylist studio + formateur (à confirmer)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>YASSINE</t>
+          <t>OLIVIER</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yassine 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et ce que vous transmettez, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YASSINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Olivier 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers hairstyle, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OLIVIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>@mathino_barber</t>
+          <t>@yassine.jarrar</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>22 rue du Commerce, 49100 Angers</t>
+          <t>21 Parvis Saint-Maurice, 59000 Lille</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MN Barbershop</t>
+          <t>Les Vilains Barber</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Barbier + formateur</t>
+          <t>Barbier + formateur (LVB Formation)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MATHINO</t>
+          <t>YASSINE</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mathino 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Yassine 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et ce que vous transmettez, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YASSINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>@hommepur_barbershop</t>
+          <t>@mathino_barber</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1044 Chemin des Plantades, 83130 La Garde</t>
+          <t>22 rue du Commerce, 49100 Angers</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Homme Pur Barber Shop</t>
+          <t>MN Barbershop</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1071,458 +1071,490 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>JABRANE</t>
+          <t>MATHINO</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jabrane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et vos soins, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JABRANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Mathino 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>@angeliquefournial</t>
+          <t>@hommepur_barbershop</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>45 Résidence des Pyrénées, 31130 Balma</t>
+          <t>1044 Chemin des Plantades, 83130 La Garde</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AF Beauté</t>
+          <t>Homme Pur Barber Shop</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Maquillage permanent / cils + formatrice</t>
+          <t>Barbier + formateur</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ANGELIQUE</t>
+          <t>JABRANE</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Angélique 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du maquillage permanent, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ANGELIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jabrane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et vos soins, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JABRANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>@chenetyelena</t>
+          <t>@angeliquefournial</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Impasse des Pins, 69003 Lyon</t>
+          <t>45 Résidence des Pyrénées, 31130 Balma</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lyon Manucure</t>
+          <t>AF Beauté</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Prothésiste ongulaire + formatrice</t>
+          <t>Maquillage permanent / cils + formatrice</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>YELENA</t>
+          <t>ANGELIQUE</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yelena 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail en onglerie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YELENA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Angélique 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du maquillage permanent, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ANGELIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>@nalhya_academy</t>
+          <t>@chenetyelena</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>34 rue de Lille, 59250 Halluin</t>
+          <t>Impasse des Pins, 69003 Lyon</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nalhya Academy</t>
+          <t>Lyon Manucure</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Cils / onglerie / esthétique + formatrice</t>
+          <t>Prothésiste ongulaire + formatrice</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>NALHYA</t>
+          <t>YELENA</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Emilie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail autour de la beauté du regard, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est NALHYA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Yelena 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail en onglerie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YELENA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>@beautycils.rennes</t>
+          <t>@nalhya_academy</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4 Bd d'Émeraude, 35760 Montgermont</t>
+          <t>34 rue de Lille, 59250 Halluin</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BeautyCils Rennes</t>
+          <t>Nalhya Academy</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Extensions de cils + formatrice</t>
+          <t>Cils / onglerie / esthétique + formatrice</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SOAZIG</t>
+          <t>NALHYA</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Soazig 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail autour du regard, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SOAZIG. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Emilie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail autour de la beauté du regard, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est NALHYA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>@beau.tynails51 (à confirmer)</t>
+          <t>@beautycils.rennes</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2A Av. Roger Martin du Gard, 51430 Tinqueux</t>
+          <t>4 Bd d'Émeraude, 35760 Montgermont</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Beauty&amp;Nail's</t>
+          <t>BeautyCils Rennes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Prothésiste ongulaire + formatrice</t>
+          <t>Extensions de cils + formatrice</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LAURA</t>
+          <t>SOAZIG</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Laura 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail en onglerie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LAURA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Soazig 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail autour du regard, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SOAZIG. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>@coupe.art_loic.chevert</t>
+          <t>@beau.tynails51 (à confirmer)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>22 Rue des Colonnes du Trône, 75012 Paris</t>
+          <t>2A Av. Roger Martin du Gard, 51430 Tinqueux</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Coupe Art</t>
+          <t>Beauty&amp;Nail's</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Coiffeur art de la coupe + formateur</t>
+          <t>Prothésiste ongulaire + formatrice</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LOIC</t>
+          <t>LAURA</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Loïc 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LOIC. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Laura 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail en onglerie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LAURA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>@capillary_le_salon</t>
+          <t>@coupe.art_loic.chevert</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>137 Bd Gallieni, 94120 Fontenay-sous-Bois</t>
+          <t>22 Rue des Colonnes du Trône, 75012 Paris</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Capillary Le Salon</t>
+          <t>Coupe Art</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Coloriste balayage minéral + formateur</t>
+          <t>Coiffeur art de la coupe + formateur</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CAPILLARY</t>
+          <t>LOIC</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Neshan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CAPILLARY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Loïc 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LOIC. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>@au_vingt_quatre</t>
+          <t>@capillary_le_salon</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>24 rue Montorgueil, 75001 Paris</t>
+          <t>137 Bd Gallieni, 94120 Fontenay-sous-Bois</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Au Vingt-Quatre</t>
+          <t>Capillary Le Salon</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Coloriste expert blond + formateur (proprio à confirmer)</t>
+          <t>Coloriste balayage minéral + formateur</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>JORIS</t>
+          <t>CAPILLARY</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Joris 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORIS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Neshan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CAPILLARY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>@bouclesdebene_studio</t>
+          <t>@au_vingt_quatre</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3 Avenue Henri Ravera, 92220 Bagneux</t>
+          <t>24 rue Montorgueil, 75001 Paris</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Boucles d'Ebène Studio</t>
+          <t>Au Vingt-Quatre</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Spécialiste cheveux bouclés/crépus + formatrice</t>
+          <t>Coloriste expert blond + formateur (proprio à confirmer)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ALINE</t>
+          <t>JORIS</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Aline 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux bouclés et crépus, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ALINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Joris 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORIS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>@cfb.studio</t>
+          <t>@bouclesdebene_studio</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>19 Rue de Stockholm, 77144 Montévrain</t>
+          <t>3 Avenue Henri Ravera, 92220 Bagneux</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CFB Studio</t>
+          <t>Boucles d'Ebène Studio</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Spécialiste cheveux crépus/frisés + formatrice</t>
+          <t>Spécialiste cheveux bouclés/crépus + formatrice</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CFB</t>
+          <t>ALINE</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Owen 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CFB. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Aline 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux bouclés et crépus, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ALINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>@labarbieredeparis</t>
+          <t>@cfb.studio</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7 rue Bertin Poirée, 75001 Paris</t>
+          <t>19 Rue de Stockholm, 77144 Montévrain</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>La Barbière de Paris</t>
+          <t>CFB Studio</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Barbier (1re femme barbier de France) + académie</t>
+          <t>Spécialiste cheveux crépus/frisés + formatrice</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SARAHH</t>
+          <t>CFB</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours unique de barbière et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Owen 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CFB. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>@maigastudio</t>
+          <t>@labarbieredeparis</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25 Rue d'Ariane, 77700 Chessy</t>
+          <t>7 rue Bertin Poirée, 75001 Paris</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Maïga Studio</t>
+          <t>La Barbière de Paris</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Coloriste cheveux texturés + formatrice</t>
+          <t>Barbier (1re femme barbier de France) + académie</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>MAIGA</t>
+          <t>SARAHH</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Halimatou 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés et votre école, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MAIGA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours unique de barbière et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>@sandrasabina31</t>
+          <t>@maigastudio</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>12 Avenue de l'Europe, Villa San Diego, 31520 Ramonville-Saint-Agne</t>
+          <t>25 Rue d'Ariane, 77700 Chessy</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Sandra Sabina</t>
+          <t>Maïga Studio</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Maquillage permanent / dermopigmentation + formatrice</t>
+          <t>Coloriste cheveux texturés + formatrice</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SANDRA</t>
+          <t>MAIGA</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sandra 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du maquillage permanent, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SANDRA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Halimatou 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés et votre école, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MAIGA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>@sandrasabina31</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12 Avenue de l'Europe, Villa San Diego, 31520 Ramonville-Saint-Agne</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sandra Sabina</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Maquillage permanent / dermopigmentation + formatrice</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SANDRA</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour Sandra 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du maquillage permanent, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SANDRA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>@casa__barbershop</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>14 Rue Romarin, 69001 Lyon</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Casa Barbershop</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Barbier + Casa Académie (gérants/fondateurs)</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>CASA</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Bonjour 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et la Casa Académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CASA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>

</xml_diff>

<commit_message>
Swap home-only Jessica for Jessica Maury (salon owner in Tours)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -603,22 +603,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>@jessicalacoiffureatonimage</t>
+          <t>@atelier_jessica_maury</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>52 Chemin des Rousselles, 69640 Lacenas (à domicile)</t>
+          <t>39 Rue Marceau, 37000 Tours</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>La Coiffure à ton image</t>
+          <t>Atelier Jessica Maury (l'atelier d'argan)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Coiffeuse-maquilleuse mariée À DOMICILE + formatrice (déjà contactée)</t>
+          <t>Coiffeuse coloriste végétale / gérante (équipe de 5)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers coiffure et maquillage mariée, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre approche végétale, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adapt Graziella message: institut de formation, no client salon
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -650,7 +650,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Coiffeuse + directrice/formatrice</t>
+          <t>Formatrice coiffure (institut de formation — pas de salon client)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Graziella 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours et votre travail de formatrice, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est GRAZIELLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Graziella 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours et votre travail de formatrice, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet aux clients d'un salon de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement et, si le cœur vous en dit, présentez-le aux coiffeurs que vous formez, sans aucune obligation. Votre code personnel est GRAZIELLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refocus seeding list on large salons with formation/academy (26 contacts)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -507,1054 +507,798 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>@cecilemollondeschamps</t>
+          <t>@sarah_pavlovski</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>221 rue Saint-Jacques, 75005 Paris</t>
+          <t>24 rue Montorgueil, 75001 Paris</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5e Caractère</t>
+          <t>Salon Sarah Pavlovski</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Coiffeuse coupe + formatrice MasterCut</t>
+          <t>Coiffeuse-coloriste cheveux texturés + formatrice</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CECILE</t>
+          <t>SARAHP</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Cécile 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CECILE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHP. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>@sarah_pavlovski</t>
+          <t>@lesalonvagabond</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>24 rue Montorgueil, 75001 Paris</t>
+          <t>4 Grand Rue, 34725 Saint-André-de-Sangonis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Salon Sarah Pavlovski</t>
+          <t>Le Salon Vagabond</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Coiffeuse-coloriste cheveux texturés + formatrice</t>
+          <t>Coloriste blond polaire / balayage + formatrice</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SARAHP</t>
+          <t>VAGABOND</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHP. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Marion 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond polaire et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est VAGABOND. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>@lesalonvagabond</t>
+          <t>@atelier_jessica_maury</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4 Grand Rue, 34725 Saint-André-de-Sangonis</t>
+          <t>39 Rue Marceau, 37000 Tours</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Le Salon Vagabond</t>
+          <t>Atelier Jessica Maury (l'atelier d'argan)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Coloriste blond polaire / balayage + formatrice</t>
+          <t>Coiffeuse coloriste végétale / gérante (équipe de 5)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>VAGABOND</t>
+          <t>JESSICA</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Marion 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond polaire et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est VAGABOND. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre approche végétale, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>@atelier_jessica_maury</t>
+          <t>@kosmocut_hairstyl (à confirmer)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>39 Rue Marceau, 37000 Tours</t>
+          <t>20 rue de l'Horloge, 63200 Riom</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Atelier Jessica Maury (l'atelier d'argan)</t>
+          <t>Synergie Coiffure Esthétique</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Coiffeuse coloriste végétale / gérante (équipe de 5)</t>
+          <t>Coiffeuse championne du monde + formatrice</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JESSICA</t>
+          <t>LISA</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre approche végétale, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>@formation.graziella.debousse</t>
+          <t>@oceaneavakian</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28 allée CF Justin Josserand, 26200 Montélimar</t>
+          <t>32 rue Cuvier, 69006 Lyon</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Institut de Formation GD</t>
+          <t>Salon Océane Avakian</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Formatrice coiffure (institut de formation — pas de salon client)</t>
+          <t>Coloriste balayage + formatrice</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GRAZIELLA</t>
+          <t>OCEANE</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Graziella 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours et votre travail de formatrice, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet aux clients d'un salon de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement et, si le cœur vous en dit, présentez-le aux coiffeurs que vous formez, sans aucune obligation. Votre code personnel est GRAZIELLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Océane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et vos formations, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OCEANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>@kosmocut_hairstyl (à confirmer)</t>
+          <t>@thomastuccinardi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>20 rue de l'Horloge, 63200 Riom</t>
+          <t>39 rue de la République, 69002 Lyon</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Synergie Coiffure Esthétique</t>
+          <t>Thomas Tuccinardi</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Coiffeuse championne du monde + formatrice</t>
+          <t>Coloriste expert + formateur (Redken)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LISA</t>
+          <t>THOMAS</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Thomas 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>@oceaneavakian</t>
+          <t>@yohanmenzoyan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>32 rue Cuvier, 69006 Lyon</t>
+          <t>37 Corniche de Solviou, 83140 Six-Fours-les-Plages</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Salon Océane Avakian</t>
+          <t>The Hairdresser</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Coloriste balayage + formatrice</t>
+          <t>Coiffeur/gérant + formateur</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OCEANE</t>
+          <t>YOHAN</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Océane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et vos formations, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OCEANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Yohan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre vision du métier et vos salons, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YOHAN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>@thomastuccinardi</t>
+          <t>@backstage_by_karatas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>39 rue de la République, 69002 Lyon</t>
+          <t>89 rue des Grandes Arcades, 67000 Strasbourg</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thomas Tuccinardi</t>
+          <t>Backstage by Karatas</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Coloriste expert + formateur (Redken)</t>
+          <t>Coloriste balayage/blond + formatrice (ALSACE)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>THOMAS</t>
+          <t>AYLA</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Thomas 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Ayla 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est AYLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>@yohanmenzoyan</t>
+          <t>@sibelhairartist</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>37 Corniche de Solviou, 83140 Six-Fours-les-Plages</t>
+          <t>14 Avenue de Strasbourg, 67170 Brumath</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The Hairdresser</t>
+          <t>Sibel Hair Artist</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Coiffeur/gérant + formateur</t>
+          <t>Coloriste balayage + formatrice (ALSACE)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>YOHAN</t>
+          <t>SIBEL</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yohan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre vision du métier et vos salons, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YOHAN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sibel 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SIBEL. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>@backstage_by_karatas</t>
+          <t>@lamaisonducoloriste</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>89 rue des Grandes Arcades, 67000 Strasbourg</t>
+          <t>18 rue des Ponts de Comines, 59800 Lille</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Backstage by Karatas</t>
+          <t>La Maison du Coloriste</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Coloriste balayage/blond + formatrice (ALSACE)</t>
+          <t>Coloriste + formateur</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>AYLA</t>
+          <t>SEBASTIEN</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Ayla 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est AYLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sébastien 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre approche du métier de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SEBASTIEN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>@sibelhairartist</t>
+          <t>@l.atypique</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14 Avenue de Strasbourg, 67170 Brumath</t>
+          <t>16 rue Littré, 75006 Paris</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sibel Hair Artist</t>
+          <t>L.Atypique</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Coloriste balayage + formatrice (ALSACE)</t>
+          <t>Coloriste blond/balayage + formatrice</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SIBEL</t>
+          <t>LATYPIQUE</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sibel 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SIBEL. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Mélanie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LATYPIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>@lamaisonducoloriste</t>
+          <t>@brookelynbalayage</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>18 rue des Ponts de Comines, 59800 Lille</t>
+          <t>9 Place Carnot, 69002 Lyon</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>La Maison du Coloriste</t>
+          <t>CL Concept</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Coloriste + formateur</t>
+          <t>Coloriste AirTouch + formatrice</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEBASTIEN</t>
+          <t>BROOKELYN</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sébastien 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre approche du métier de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SEBASTIEN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour BrookeLyn 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du balayage AirTouch, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est BROOKELYN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>@l.atypique</t>
+          <t>@salon_kf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16 rue Littré, 75006 Paris</t>
+          <t>69 Bd Ernest Dalby, 44000 Nantes</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>L.Atypique</t>
+          <t>Salon KF</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Coloriste blond/balayage + formatrice</t>
+          <t>Coiffeur coloriste + formateur</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LATYPIQUE</t>
+          <t>SALONKF</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mélanie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LATYPIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Kévin 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SALONKF. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>@brookelynbalayage</t>
+          <t>@olivierlebrun_paris</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>9 Place Carnot, 69002 Lyon</t>
+          <t>5 bis rue du Louvre, 75001 Paris</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CL Concept</t>
+          <t>OLAB Paris</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Coloriste AirTouch + formatrice</t>
+          <t>Hairstylist studio + formateur (à confirmer)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BROOKELYN</t>
+          <t>OLIVIER</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Bonjour BrookeLyn 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du balayage AirTouch, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est BROOKELYN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Olivier 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers hairstyle, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OLIVIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>@salon_kf</t>
+          <t>@yassine.jarrar</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>69 Bd Ernest Dalby, 44000 Nantes</t>
+          <t>21 Parvis Saint-Maurice, 59000 Lille</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Salon KF</t>
+          <t>Les Vilains Barber</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Coiffeur coloriste + formateur</t>
+          <t>Barbier + formateur (LVB Formation)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SALONKF</t>
+          <t>YASSINE</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Kévin 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SALONKF. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Yassine 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et ce que vous transmettez, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YASSINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>@olivierlebrun_paris</t>
+          <t>@mathino_barber</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5 bis rue du Louvre, 75001 Paris</t>
+          <t>22 rue du Commerce, 49100 Angers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OLAB Paris</t>
+          <t>MN Barbershop</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hairstylist studio + formateur (à confirmer)</t>
+          <t>Barbier + formateur</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OLIVIER</t>
+          <t>MATHINO</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Olivier 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers hairstyle, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OLIVIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Mathino 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>@yassine.jarrar</t>
+          <t>@hommepur_barbershop</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>21 Parvis Saint-Maurice, 59000 Lille</t>
+          <t>1044 Chemin des Plantades, 83130 La Garde</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Les Vilains Barber</t>
+          <t>Homme Pur Barber Shop</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Barbier + formateur (LVB Formation)</t>
+          <t>Barbier + formateur</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YASSINE</t>
+          <t>JABRANE</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yassine 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et ce que vous transmettez, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YASSINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jabrane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et vos soins, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JABRANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>@mathino_barber</t>
+          <t>@coupe.art_loic.chevert</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>22 rue du Commerce, 49100 Angers</t>
+          <t>22 Rue des Colonnes du Trône, 75012 Paris</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MN Barbershop</t>
+          <t>Coupe Art</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Barbier + formateur</t>
+          <t>Coiffeur art de la coupe + formateur</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MATHINO</t>
+          <t>LOIC</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mathino 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Loïc 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LOIC. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>@hommepur_barbershop</t>
+          <t>@capillary_le_salon</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1044 Chemin des Plantades, 83130 La Garde</t>
+          <t>137 Bd Gallieni, 94120 Fontenay-sous-Bois</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Homme Pur Barber Shop</t>
+          <t>Capillary Le Salon</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Barbier + formateur</t>
+          <t>Coloriste balayage minéral + formateur</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>JABRANE</t>
+          <t>CAPILLARY</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jabrane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et vos soins, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JABRANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Neshan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CAPILLARY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>@angeliquefournial</t>
+          <t>@au_vingt_quatre</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>45 Résidence des Pyrénées, 31130 Balma</t>
+          <t>24 rue Montorgueil, 75001 Paris</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AF Beauté</t>
+          <t>Au Vingt-Quatre</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Maquillage permanent / cils + formatrice</t>
+          <t>Coloriste expert blond + formateur (proprio à confirmer)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ANGELIQUE</t>
+          <t>JORIS</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Angélique 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du maquillage permanent, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ANGELIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Joris 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORIS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>@chenetyelena</t>
+          <t>@bouclesdebene_studio</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Impasse des Pins, 69003 Lyon</t>
+          <t>3 Avenue Henri Ravera, 92220 Bagneux</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Lyon Manucure</t>
+          <t>Boucles d'Ebène Studio</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Prothésiste ongulaire + formatrice</t>
+          <t>Spécialiste cheveux bouclés/crépus + formatrice</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YELENA</t>
+          <t>ALINE</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yelena 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail en onglerie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YELENA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Aline 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux bouclés et crépus, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ALINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>@nalhya_academy</t>
+          <t>@cfb.studio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>34 rue de Lille, 59250 Halluin</t>
+          <t>19 Rue de Stockholm, 77144 Montévrain</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nalhya Academy</t>
+          <t>CFB Studio</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cils / onglerie / esthétique + formatrice</t>
+          <t>Spécialiste cheveux crépus/frisés + formatrice</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NALHYA</t>
+          <t>CFB</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Emilie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail autour de la beauté du regard, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est NALHYA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Owen 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CFB. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>@beautycils.rennes</t>
+          <t>@labarbieredeparis</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4 Bd d'Émeraude, 35760 Montgermont</t>
+          <t>7 rue Bertin Poirée, 75001 Paris</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BeautyCils Rennes</t>
+          <t>La Barbière de Paris</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Extensions de cils + formatrice</t>
+          <t>Barbier (1re femme barbier de France) + académie</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SOAZIG</t>
+          <t>SARAHH</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Soazig 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail autour du regard, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SOAZIG. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours unique de barbière et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>@beau.tynails51 (à confirmer)</t>
+          <t>@maigastudio</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2A Av. Roger Martin du Gard, 51430 Tinqueux</t>
+          <t>25 Rue d'Ariane, 77700 Chessy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Beauty&amp;Nail's</t>
+          <t>Maïga Studio</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Prothésiste ongulaire + formatrice</t>
+          <t>Coloriste cheveux texturés + formatrice</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LAURA</t>
+          <t>MAIGA</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Laura 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail en onglerie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LAURA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Halimatou 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés et votre école, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MAIGA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>@coupe.art_loic.chevert</t>
+          <t>@casa__barbershop</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>22 Rue des Colonnes du Trône, 75012 Paris</t>
+          <t>14 Rue Romarin, 69001 Lyon</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Coupe Art</t>
+          <t>Casa Barbershop</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Coiffeur art de la coupe + formateur</t>
+          <t>Barbier + Casa Académie (gérants/fondateurs)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LOIC</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Loïc 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LOIC. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>@capillary_le_salon</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>137 Bd Gallieni, 94120 Fontenay-sous-Bois</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Capillary Le Salon</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Coloriste balayage minéral + formateur</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>CAPILLARY</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Neshan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CAPILLARY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>@au_vingt_quatre</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>24 rue Montorgueil, 75001 Paris</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Au Vingt-Quatre</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Coloriste expert blond + formateur (proprio à confirmer)</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>JORIS</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Joris 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORIS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>@bouclesdebene_studio</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>3 Avenue Henri Ravera, 92220 Bagneux</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Boucles d'Ebène Studio</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Spécialiste cheveux bouclés/crépus + formatrice</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ALINE</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Aline 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux bouclés et crépus, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ALINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>@cfb.studio</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>19 Rue de Stockholm, 77144 Montévrain</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>CFB Studio</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Spécialiste cheveux crépus/frisés + formatrice</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>CFB</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Owen 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CFB. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>@labarbieredeparis</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>7 rue Bertin Poirée, 75001 Paris</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>La Barbière de Paris</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Barbier (1re femme barbier de France) + académie</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>SARAHH</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours unique de barbière et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>@maigastudio</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>25 Rue d'Ariane, 77700 Chessy</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Maïga Studio</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Coloriste cheveux texturés + formatrice</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>MAIGA</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Halimatou 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés et votre école, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MAIGA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>@sandrasabina31</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>12 Avenue de l'Europe, Villa San Diego, 31520 Ramonville-Saint-Agne</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Sandra Sabina</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Maquillage permanent / dermopigmentation + formatrice</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>SANDRA</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour Sandra 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du maquillage permanent, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SANDRA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>@casa__barbershop</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>14 Rue Romarin, 69001 Lyon</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Casa Barbershop</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Barbier + Casa Académie (gérants/fondateurs)</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>CASA</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Bonjour 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et la Casa Académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CASA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>

</xml_diff>

<commit_message>
Multi-salon: one row per location, neutral greeting, add sans abonnement to messages
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jordy 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur les extensions et la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORDY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jordy 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur les extensions et la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORDY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Coiffeuse-coloriste cheveux texturés + formatrice</t>
+          <t>Coiffeuse-coloriste cheveux texturés + formatrice (multi-salons : autres adresses à confirmer)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHP. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAHP. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Marion 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond polaire et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est VAGABOND. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Marion 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond polaire et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est VAGABOND. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre approche végétale, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jessica 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre approche végétale, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JESSICA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Océane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et vos formations, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OCEANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Océane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et vos formations, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OCEANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Thomas 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Coiffeur/gérant + formateur</t>
+          <t>Coiffeur/gérant + formateur (multi-salons : autres adresses à confirmer)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yohan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre vision du métier et vos salons, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YOHAN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est YOHAN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Ayla 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est AYLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Ayla 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond et le balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est AYLA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sibel 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SIBEL. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sibel 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du balayage, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SIBEL. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sébastien 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre approche du métier de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SEBASTIEN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Sébastien 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre approche du métier de coloriste, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SEBASTIEN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mélanie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LATYPIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Mélanie 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail sur le blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LATYPIQUE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Bonjour BrookeLyn 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du balayage AirTouch, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est BROOKELYN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour BrookeLyn 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre maîtrise du balayage AirTouch, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est BROOKELYN. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Kévin 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SALONKF. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Kévin 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SALONKF. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Olivier 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers hairstyle, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OLIVIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Olivier 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers hairstyle, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est OLIVIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Barbier + formateur (LVB Formation)</t>
+          <t>Barbier + formateur (LVB Formation) (multi-salons : autres adresses à confirmer)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Yassine 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et ce que vous transmettez, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est YASSINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est YASSINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mathino 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Jabrane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et vos soins, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JABRANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Jabrane 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et vos soins, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JABRANE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Loïc 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LOIC. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Loïc 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre art de la coupe, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LOIC. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Neshan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CAPILLARY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Neshan 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre travail de coloriste et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CAPILLARY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Joris 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORIS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Joris 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise du blond, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est JORIS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Aline 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux bouclés et crépus, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ALINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Aline 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux bouclés et crépus, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est ALINE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Owen 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CFB. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Owen 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CFB. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Sarah 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours unique de barbière et votre académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Halimatou 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés et votre école, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MAIGA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour Halimatou 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre expertise des cheveux texturés et votre école, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est MAIGA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,231 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Bonjour 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et la Casa Académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CASA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre univers barbier et la Casa Académie, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est CASA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>@thomastuccinardi</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>26 rue Étienne Marcel, 75002 Paris</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Thomas Tuccinardi</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Coloriste expert + formateur (Redken)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>THOMAS</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est THOMAS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>@mathino_barber</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>29 Rue Georges Clemenceau, 49300 Cholet</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MN Barbershop</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Barbier + formateur</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MATHINO</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>@mathino_barber</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>18 Rue Beaurepaire, 49400 Saumur</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MN Barbershop</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Barbier + formateur</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MATHINO</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>@mathino_barber</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20 Rue Pasteur, 49500 Segré-en-Anjou Bleu</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MN Barbershop</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Barbier + formateur</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MATHINO</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MATHINO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>@labarbieredeparis</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>21 rue Condorcet, 75009 Paris</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>La Barbière de Paris</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Barbier (1re femme barbier de France) + académie</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SARAHH</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>@labarbieredeparis</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>19 rue de l'Abbé Grégoire, 75006 Paris</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>La Barbière de Paris</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Barbier (1re femme barbier de France) + académie</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SARAHH</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>@labarbieredeparis</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>37 bd des Capucines, 75002 Paris</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>La Barbière de Paris</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Barbier (1re femme barbier de France) + académie</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SARAHH</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAHH. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 10 large salons with academies (KMS, Les Garcons Barbiers, Medley, Saco, etc.)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1528,6 +1528,326 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>@kmsbarber</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>127 rue Fondaudège, 33000 Bordeaux</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KMS Barber</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Barbershop (7 salons) + KMS Barber Academy (multi-salons : autres adresses à confirmer)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>KMS</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est KMS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>@lesgarconsbarbiers</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>13 rue Saint-Lazare, 75009 Paris</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Les Garçons Barbiers</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Barbershop réseau Paris (~7 salons) + Barber Academy (multi-salons : autres adresses à confirmer)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>GARCONS</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est GARCONS. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>@medley.marais</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>21 rue Vieille du Temple, 75004 Paris</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Medley (Rive Droite)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Salon coiffure haut de gamme + Medley Academy (stages Wella)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MEDLEY</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MEDLEY. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>@sacofrance</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>78 rue du Loup, 33000 Bordeaux</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Saco France</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Salon coiffure + académie de formation (ambassadeur Schwarzkopf)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SACO</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SACO. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>@eleganceacademie</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19 boulevard d'Arcole, 31000 Toulouse</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Élégance Académie</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Salon coiffure mixte + centre de formation</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ELEGANCE</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est ELEGANCE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>@barberlacrim75</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>53 rue d'Avron, 75020 Paris</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>The Barber by Lacrim</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Barbershop réseau (8 salons) + formation (multi-salons : autres adresses à confirmer)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LACRIM</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est LACRIM. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>@latelierdubarbierofficiel</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10 bd de la Prairie au Duc, 44200 Nantes</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>L'Atelier du Barbier</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Barbershop (6 salons Nantes) + formation (multi-salons : autres adresses à confirmer)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ATELIERBARBIER</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est ATELIERBARBIER. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>@freshcut.nantes</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Carré Feydeau, 1 Cours Cdt d'Estienne d'Orves, 44000 Nantes</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>FreshCut BarberShop</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Barbershop (3-4 salons) + section formation (multi-salons : autres adresses à confirmer)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FRESHCUT</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est FRESHCUT. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>@lecuriedubarber</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>21 rue de la Mare de Troux, 78280 Guyancourt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>L'Écurie du Barber</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Barbershop + centre de formation barbiers</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ECURIE</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est ECURIE. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>@franckprovostofficiel</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>36 rue Laugier, 75017 Paris</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Académie Franck Provost</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Grand salon + académie internationale (handle = compte marque, à confirmer)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PROVOST</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est PROVOST. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Synergie Coiffure: new 2025 address + neutral team greeting
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20 rue de l'Horloge, 63200 Riom</t>
+          <t>29 rue de l'Hôtel de Ville, 63200 Riom (déménagé 2025 — vérifier)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Coiffeuse championne du monde + formatrice</t>
+          <t>Salon Synergie (gérante Lisa Derossis, championne du monde 2019 + formatrice) — équipe</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Lisa 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. J'admire vraiment votre parcours de championne du monde, et je me suis dit que vous étiez exactement la bonne personne pour le découvrir. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner aux équipes ce que la disparition du liquide leur fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans votre salon, sans aucune obligation. Et si un jour vous avez envie de le partager autour de vous, votre code personnel est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Raphaël, le fondateur de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est LISA. Un immense merci, et très belle journée à vous. Raphaël — digitip.app</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Tuccinardi Paris salon as separate seeding row
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1324,14 +1324,62 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>@thomastuccinardi</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>26 rue Étienne Marcel, 75002 Paris</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Thomas Tuccinardi</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Coloriste expert + formateur (académie, Redken)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>THOMAS10</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est THOMAS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>À envoyer</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>À préparer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="G2:G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À envoyer,Envoyé,Réponse reçue,Intéressé,Partenaire,Refus"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À préparer,Envoyé,Activé,Non activé"</formula1>
     </dataValidation>
+    <dataValidation sqref="G2:G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"À envoyer,Envoyé,Réponse reçue,Intéressé,Partenaire,Refus"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"À préparer,Envoyé,Activé,Non activé"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove BrookeLyn (solo, not salon owner) from seeding list
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -781,32 +781,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>@brookelynbalayage</t>
+          <t>@jordy.brechkoff</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9 Place Carnot, 69002 Lyon</t>
+          <t>135 bd Haussmann, 75008 Paris</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CL Concept</t>
+          <t>Jordy Brechkoff</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Coloriste AirTouch + formatrice (masterclass)</t>
+          <t>Coiffeur extensions + formateur (masterclass)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BROOKELYN10</t>
+          <t>JORDY10</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est BROOKELYN10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est JORDY10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -823,32 +823,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>@jordy.brechkoff</t>
+          <t>@sarah_pavlovski</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>135 bd Haussmann, 75008 Paris</t>
+          <t>24 rue Montorgueil, 75001 Paris</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jordy Brechkoff</t>
+          <t>Salon Sarah Pavlovski</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Coiffeur extensions + formateur (masterclass)</t>
+          <t>Coiffeuse-coloriste cheveux texturés + formation</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>JORDY10</t>
+          <t>SARAH10</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est JORDY10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAH10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -865,32 +865,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>@sarah_pavlovski</t>
+          <t>@olivierlebrun_paris</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>24 rue Montorgueil, 75001 Paris</t>
+          <t>5 bis rue du Louvre, 75001 Paris</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Salon Sarah Pavlovski</t>
+          <t>OLAB Paris</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Coiffeuse-coloriste cheveux texturés + formation</t>
+          <t>Hairstylist studio + formateur</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SARAH10</t>
+          <t>OLAB10</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SARAH10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est OLAB10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -907,32 +907,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>@olivierlebrun_paris</t>
+          <t>@yassine.jarrar</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5 bis rue du Louvre, 75001 Paris</t>
+          <t>21 Parvis Saint-Maurice, 59000 Lille</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OLAB Paris</t>
+          <t>Les Vilains Barber</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Hairstylist studio + formateur</t>
+          <t>Barbershop (3 salons) + LVB Formation</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OLAB10</t>
+          <t>VILAINS10</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est OLAB10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est VILAINS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -949,32 +949,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>@yassine.jarrar</t>
+          <t>@mathino_barber</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21 Parvis Saint-Maurice, 59000 Lille</t>
+          <t>22 rue du Commerce, 49100 Angers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Les Vilains Barber</t>
+          <t>MN Barbershop</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Barbershop (3 salons) + LVB Formation</t>
+          <t>Barbershop (4 salons) + formation</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>VILAINS10</t>
+          <t>MNBARBER10</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est VILAINS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MNBARBER10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -991,32 +991,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>@mathino_barber</t>
+          <t>@hommepur_barbershop</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>22 rue du Commerce, 49100 Angers</t>
+          <t>1044 Chemin des Plantades, 83130 La Garde</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MN Barbershop</t>
+          <t>Homme Pur Barber Shop</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Barbershop (4 salons) + formation</t>
+          <t>Barbershop + centre de formation</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MNBARBER10</t>
+          <t>HOMMEPUR10</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MNBARBER10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est HOMMEPUR10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1033,32 +1033,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>@hommepur_barbershop</t>
+          <t>@labarbieredeparis</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1044 Chemin des Plantades, 83130 La Garde</t>
+          <t>7 rue Bertin Poirée, 75001 Paris</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Homme Pur Barber Shop</t>
+          <t>La Barbière de Paris</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Barbershop + centre de formation</t>
+          <t>Barbershop (6 salons) + académie</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HOMMEPUR10</t>
+          <t>BARBIERE10</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est HOMMEPUR10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est BARBIERE10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1075,32 +1075,32 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>@labarbieredeparis</t>
+          <t>@kmsbarber</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7 rue Bertin Poirée, 75001 Paris</t>
+          <t>127 rue Fondaudège, 33000 Bordeaux</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>La Barbière de Paris</t>
+          <t>KMS Barber</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Barbershop (6 salons) + académie</t>
+          <t>Barbershop (7 salons) + KMS Barber Academy</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BARBIERE10</t>
+          <t>KMS10</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est BARBIERE10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est KMS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1117,32 +1117,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>@kmsbarber</t>
+          <t>@lesgarconsbarbiers</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>127 rue Fondaudège, 33000 Bordeaux</t>
+          <t>13 rue Saint-Lazare, 75009 Paris</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KMS Barber</t>
+          <t>Les Garçons Barbiers</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Barbershop (7 salons) + KMS Barber Academy</t>
+          <t>Barbershop réseau Paris + Barber Academy</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>KMS10</t>
+          <t>GARCONS10</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est KMS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est GARCONS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1159,32 +1159,32 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>@lesgarconsbarbiers</t>
+          <t>@medley.marais</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>13 rue Saint-Lazare, 75009 Paris</t>
+          <t>21 rue Vieille du Temple, 75004 Paris</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Les Garçons Barbiers</t>
+          <t>Medley (Rive Droite)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Barbershop réseau Paris + Barber Academy</t>
+          <t>Salon haut de gamme + Medley Academy (Wella)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GARCONS10</t>
+          <t>MEDLEY10</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est GARCONS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MEDLEY10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1201,32 +1201,32 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>@medley.marais</t>
+          <t>@sacofrance</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>21 rue Vieille du Temple, 75004 Paris</t>
+          <t>78 rue du Loup, 33000 Bordeaux</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Medley (Rive Droite)</t>
+          <t>Saco France</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Salon haut de gamme + Medley Academy (Wella)</t>
+          <t>Salon + académie de formation (Schwarzkopf)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MEDLEY10</t>
+          <t>SACO10</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est MEDLEY10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SACO10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1243,32 +1243,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>@sacofrance</t>
+          <t>@eleganceacademie</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>78 rue du Loup, 33000 Bordeaux</t>
+          <t>19 boulevard d'Arcole, 31000 Toulouse</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Saco France</t>
+          <t>Élégance Académie</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Salon + académie de formation (Schwarzkopf)</t>
+          <t>Salon coiffure + centre de formation</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SACO10</t>
+          <t>ELEGANCE10</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est SACO10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est ELEGANCE10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1285,32 +1285,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>@eleganceacademie</t>
+          <t>@thomastuccinardi</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>19 boulevard d'Arcole, 31000 Toulouse</t>
+          <t>26 rue Étienne Marcel, 75002 Paris</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Élégance Académie</t>
+          <t>Thomas Tuccinardi</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Salon coiffure + centre de formation</t>
+          <t>Coloriste expert + formateur (académie, Redken)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ELEGANCE10</t>
+          <t>THOMAS10</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est ELEGANCE10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
+          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est THOMAS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1319,48 +1319,6 @@
         </is>
       </c>
       <c r="H21" t="inlineStr">
-        <is>
-          <t>À préparer</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>@thomastuccinardi</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>26 rue Étienne Marcel, 75002 Paris</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Thomas Tuccinardi</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Coloriste expert + formateur (académie, Redken)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>THOMAS10</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Bonjour à toute l'équipe 🙂 Je suis Océane, la fondatrice de Digitip, et c'est avec un grand plaisir que je vous offre ce petit tag. C'est une petite plaque sans contact qui permet à vos clients de laisser un pourboire en quelques secondes, sans espèces, pour redonner à l'équipe ce que la disparition du liquide lui fait perdre. C'est un achat unique, sans abonnement. Testez-le tranquillement dans le salon, sans aucune obligation. Et si l'envie vous prend de le partager autour de vous, votre code est THOMAS10. Un immense merci, et très belle journée à vous. Océane — Fondatrice de Digitip — digitip.app</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>À envoyer</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>

</xml_diff>

<commit_message>
Add 2nd tab: salon business training groups to contact for demo
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Seeding Digitip - Top 20" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Formateurs business (contacter)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1341,4 +1342,320 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Organisme</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Email / Contact</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Adresse</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Focus / équipe</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>L'Atelier Accompagnement</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@latelier_accompagnement</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>contact@latelier-accompagnement.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1 rue Icare, 67960 Entzheim (ALSACE)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Équipe de 5, croissance &amp; rentabilité des salons (~150 membres)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FITBOARD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>@fitboard_official (à confirmer)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>contact@fitboard.fr</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>54 rue de Vesoul, 25000 Besançon</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Coaching dirigeants salons/instituts : pilotage, rentabilité, RH, marketing</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADR Formation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>@adrformation</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>adrformation.com/contact</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Lahosse (40), Aquitaine</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>~12 intervenants ; management &amp; développement du salon</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>APC Formation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>@apc_formation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>contact@apcformation.fr</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>5 rue Jean Dumas, 24660 Coulounieix-Chamiers</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>50+ formateurs ; RH/management/gestion/rentabilité</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Barbier Académie</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>@barbieracademie</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>contact@barbieracademie.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Paris (rue St-Honoré)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Équipe ; accompagnement 'Copilote Business' pour gérants</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ILAE Formation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>@ilaeformation</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ilaeformation.com/contact</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>non publique</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Plusieurs formateurs ; pôle gestion &amp; création d'entreprise</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wellness Consulting</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>contact@wellness-consulting.fr</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>non publique (Paris + multi-villes)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Équipe ; gestion/rentabilité — orienté spas/instituts premium</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Elegance France / Consulting</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>@elegance_academies_france</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>contact@elegance.fr</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>47 rue de l'Hôtel des Postes, 06000 Nice</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Équipe pluridisciplinaire ; consulting spa/instituts (gestion, marketing)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"À contacter,Contacté,Intéressé,Démo envoyée,Recommande,Refus"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove FITBOARD (competitor) from business training groups tab
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -1350,7 +1350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1429,27 +1429,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FITBOARD</t>
+          <t>ADR Formation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>@fitboard_official (à confirmer)</t>
+          <t>@adrformation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>contact@fitboard.fr</t>
+          <t>adrformation.com/contact</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>54 rue de Vesoul, 25000 Besançon</t>
+          <t>Lahosse (40), Aquitaine</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Coaching dirigeants salons/instituts : pilotage, rentabilité, RH, marketing</t>
+          <t>~12 intervenants ; management &amp; développement du salon</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1461,27 +1461,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADR Formation</t>
+          <t>APC Formation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>@adrformation</t>
+          <t>@apc_formation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>adrformation.com/contact</t>
+          <t>contact@apcformation.fr</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lahosse (40), Aquitaine</t>
+          <t>5 rue Jean Dumas, 24660 Coulounieix-Chamiers</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>~12 intervenants ; management &amp; développement du salon</t>
+          <t>50+ formateurs ; RH/management/gestion/rentabilité</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1493,27 +1493,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>APC Formation</t>
+          <t>Barbier Académie</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>@apc_formation</t>
+          <t>@barbieracademie</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>contact@apcformation.fr</t>
+          <t>contact@barbieracademie.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5 rue Jean Dumas, 24660 Coulounieix-Chamiers</t>
+          <t>Paris (rue St-Honoré)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>50+ formateurs ; RH/management/gestion/rentabilité</t>
+          <t>Équipe ; accompagnement 'Copilote Business' pour gérants</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1525,27 +1525,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Barbier Académie</t>
+          <t>ILAE Formation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>@barbieracademie</t>
+          <t>@ilaeformation</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>contact@barbieracademie.com</t>
+          <t>ilaeformation.com/contact</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Paris (rue St-Honoré)</t>
+          <t>non publique</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Équipe ; accompagnement 'Copilote Business' pour gérants</t>
+          <t>Plusieurs formateurs ; pôle gestion &amp; création d'entreprise</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ILAE Formation</t>
+          <t>Wellness Consulting</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>@ilaeformation</t>
+          <t>à confirmer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ilaeformation.com/contact</t>
+          <t>contact@wellness-consulting.fr</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>non publique</t>
+          <t>non publique (Paris + multi-villes)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Plusieurs formateurs ; pôle gestion &amp; création d'entreprise</t>
+          <t>Équipe ; gestion/rentabilité — orienté spas/instituts premium</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1589,62 +1589,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wellness Consulting</t>
+          <t>Elegance France / Consulting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>@elegance_academies_france</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>contact@wellness-consulting.fr</t>
+          <t>contact@elegance.fr</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>non publique (Paris + multi-villes)</t>
+          <t>47 rue de l'Hôtel des Postes, 06000 Nice</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Équipe ; gestion/rentabilité — orienté spas/instituts premium</t>
+          <t>Équipe pluridisciplinaire ; consulting spa/instituts (gestion, marketing)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
-        <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Elegance France / Consulting</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>@elegance_academies_france</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>contact@elegance.fr</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>47 rue de l'Hôtel des Postes, 06000 Nice</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Équipe pluridisciplinaire ; consulting spa/instituts (gestion, marketing)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
         <is>
           <t>À contacter</t>
         </is>

</xml_diff>

<commit_message>
Reclassify business training groups: flag technical vs pure-business
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -1417,7 +1417,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Équipe de 5, croissance &amp; rentabilité des salons (~150 membres)</t>
+          <t>✅ 100% BUSINESS : croissance &amp; rentabilité des salons (équipe de 5) — profil parfait</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>~12 intervenants ; management &amp; développement du salon</t>
+          <t>⚠️ Surtout académie TECHNIQUE + management ; volet business secondaire — à valider</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>50+ formateurs ; RH/management/gestion/rentabilité</t>
+          <t>⚠️ Surtout TECHNIQUE/RH (50+ formateurs) ; volet business secondaire — à valider</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Équipe ; accompagnement 'Copilote Business' pour gérants</t>
+          <t>⚠️ Surtout académie TECHNIQUE barbier ; petit volet 'Copilote Business'</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Équipe ; gestion/rentabilité — orienté spas/instituts premium</t>
+          <t>Business spa/instituts premium (gestion, rentabilité, taux d'occupation)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Équipe pluridisciplinaire ; consulting spa/instituts (gestion, marketing)</t>
+          <t>Consulting spa/instituts (gestion, marketing, budget)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">

</xml_diff>

<commit_message>
Add 3 pure-business salon consulting firms (Aide-Coiffure, Dont Acte, Reseau MonCoiffeur)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -1350,7 +1350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1618,6 +1618,134 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Aide-Coiffure</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>@aidecoiffure</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>formulaire aide-coiffure.fr (1re consult. gratuite)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>non publique</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>✅ 100% BUSINESS : gestion/marketing/pricing/RH des salons indépendants, équipe (consultants + comptable + CM)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DONT ACTE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dont-acte@wanadoo.fr / +33 6 83 82 41 60</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>région Rhône (à confirmer)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>✅ 100% management/business : conseil, coaching équipe, co-développement — équipe modulable</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Réseau MonCoiffeur</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>@reseaumoncoiffeur.fr</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>formulaire moncoiffeur.fr / 02 85 52 69 55</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>région Nantes (à confirmer)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>✅ BUSINESS/gestion : pilotage perf mensuel, marketing — équipe nommée (Nicolas, Clélia, Amélie…)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SRHC – SRH Consulting</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>formulaire srhconsulting.fr</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Business SPA (CA/charges, management) — plutôt spas hôtels premium (réserve)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Add 3rd tab: restaurant business coaches for resto test
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BT13qsVsMrdecpWjhKHZmW
</commit_message>
<xml_diff>
--- a/prospects_seeding_digitip.xlsx
+++ b/prospects_seeding_digitip.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Seeding Digitip - Top 20" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Formateurs business (contacter)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resto - coachs business" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +43,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007C2D12"/>
+        <bgColor rgb="007C2D12"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,13 +64,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1754,4 +1764,319 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Email / Contact</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Adresse</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Focus / type</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tomorrow Food</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@tomorrow.food</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>contact@tomorrowfood.fr / 06 82 99 54 72</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>42 rue de Paradis, 75010 Paris</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Agence 360 F&amp;B : conseil, rentabilité, concepts, ouverture — ÉQUIPE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RestHoDev (Vincent Sitz)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>formulaire resthodev.com/contact</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Paris (non publique)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Audits, gestion opé, RH, ouverture/reprise — ÉQUIPE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hôtellerie Française (Nicole Jouffret)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>@hotelleriefrancaise</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>nicole.jouffret@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>131 bis Av. de Royat, 63400 Chamalières</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Coaching gestion, management, rentabilité — solo (autrice/coach)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gira Conseil (Bernard Boutboul)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>formulaire giraconseil.fr/contact</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>non publique</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Référence du secteur depuis 1989 : stratégie/dév restauration — cabinet (groupe RYDGE)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Foodexplora (Mathieu Laville)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>@mathieu_laville</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>07 44 44 36 05 + formulaire foodexplora.fr</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>125 A route du chef lieu, 74350 Allonzier-la-Caille</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Concepts, business plans, rentabilité, audits — solo (15 ans)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vulpes Consulting (Sébastien Renard)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>@vulpesconsulting</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>formulaire vulpesconsulting.fr/contact</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>non publique</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Conseil hôtellerie/resto, audits, ouverture, gestion — solo + réseau</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NEO Engineering (Laurent Pailhès)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>à confirmer (pas d'IG)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>contact@neoeng.com / 04 91 71 35 82</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>34 avenue des Colonnes, 13008 Marseille</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Création, organisation, rentabilité resto — solo</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Digital Gourmet</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>@digital_gourmet_paris</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>formulaire digitalgourmet.fr/contact</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Paris (non publique)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Marketing/visibilité resto (social, branding) — agence (angle marketing)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"À contacter,Contacté,Intéressé,Démo envoyée,Recommande,Refus"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>